<commit_message>
updated quiz structure to match system demands
</commit_message>
<xml_diff>
--- a/quiz/old-quiz/DS1.1.xlsx
+++ b/quiz/old-quiz/DS1.1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25128"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\_5 QUESTION DATABASE\Web Database\_0 Access Database\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\firebrigade\wp-content\plugins\techiquiz\quiz\old-quiz\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4BEBDD6-1731-4027-A576-FF0C86587A66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFB658A3-DF29-4C19-A3EB-5530BD3D0008}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{965BE20A-EC08-4D90-A695-FEBB0267C9A3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{965BE20A-EC08-4D90-A695-FEBB0267C9A3}"/>
   </bookViews>
   <sheets>
     <sheet name="DS1" sheetId="10" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1759" uniqueCount="1158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1768" uniqueCount="1156">
   <si>
     <t>All the above</t>
   </si>
@@ -2152,9 +2152,6 @@
     <t>BHP will decrease slowly and increase dramatically, risking further influx.</t>
   </si>
   <si>
-    <t>Form</t>
-  </si>
-  <si>
     <t>Sign</t>
   </si>
   <si>
@@ -2243,9 +2240,6 @@
   </si>
   <si>
     <t>Gas Expansion</t>
-  </si>
-  <si>
-    <t>Answer</t>
   </si>
   <si>
     <t>Bleed off approximately 50 psi to check for trapped pressure</t>
@@ -4183,10 +4177,10 @@
         <v>243</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>759</v>
+        <v>757</v>
       </c>
       <c r="F1" s="24" t="s">
-        <v>758</v>
+        <v>756</v>
       </c>
       <c r="G1" s="13" t="s">
         <v>471</v>
@@ -4203,12 +4197,8 @@
       <c r="K1" s="13" t="s">
         <v>705</v>
       </c>
-      <c r="L1" s="13" t="s">
-        <v>707</v>
-      </c>
-      <c r="M1" s="13" t="s">
-        <v>738</v>
-      </c>
+      <c r="L1" s="13"/>
+      <c r="M1" s="13"/>
     </row>
     <row r="2" spans="1:13" s="3" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A2" s="4">
@@ -4224,7 +4214,7 @@
         <v>98</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
       <c r="F2" s="25" t="s">
         <v>296</v>
@@ -4233,7 +4223,7 @@
         <v>100</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>951</v>
+        <v>949</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>99</v>
@@ -4261,7 +4251,7 @@
         <v>106</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="F3" s="25" t="s">
         <v>274</v>
@@ -4270,7 +4260,7 @@
         <v>163</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>952</v>
+        <v>950</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>162</v>
@@ -4298,7 +4288,7 @@
         <v>106</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>762</v>
+        <v>760</v>
       </c>
       <c r="F4" s="25" t="s">
         <v>286</v>
@@ -4310,7 +4300,7 @@
         <v>252</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>953</v>
+        <v>951</v>
       </c>
       <c r="J4" s="6" t="s">
         <v>626</v>
@@ -4335,7 +4325,7 @@
         <v>106</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
       <c r="F5" s="25" t="s">
         <v>295</v>
@@ -4350,7 +4340,7 @@
         <v>634</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>954</v>
+        <v>952</v>
       </c>
       <c r="K5" s="5" t="s">
         <v>454</v>
@@ -4372,7 +4362,7 @@
         <v>42</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>764</v>
+        <v>762</v>
       </c>
       <c r="F6" s="26" t="s">
         <v>686</v>
@@ -4381,7 +4371,7 @@
         <v>49</v>
       </c>
       <c r="H6" s="12" t="s">
-        <v>994</v>
+        <v>992</v>
       </c>
       <c r="I6" s="12" t="s">
         <v>48</v>
@@ -4409,7 +4399,7 @@
         <v>149</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>765</v>
+        <v>763</v>
       </c>
       <c r="F7" s="25" t="s">
         <v>616</v>
@@ -4418,7 +4408,7 @@
         <v>159</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>995</v>
+        <v>993</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>158</v>
@@ -4446,13 +4436,13 @@
         <v>57</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="F8" s="25" t="s">
         <v>259</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>955</v>
+        <v>953</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>206</v>
@@ -4483,7 +4473,7 @@
         <v>57</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>767</v>
+        <v>765</v>
       </c>
       <c r="F9" s="25" t="s">
         <v>275</v>
@@ -4498,7 +4488,7 @@
         <v>598</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>1071</v>
+        <v>1069</v>
       </c>
       <c r="K9" s="5" t="s">
         <v>454</v>
@@ -4520,7 +4510,7 @@
         <v>57</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>768</v>
+        <v>766</v>
       </c>
       <c r="F10" s="25" t="s">
         <v>273</v>
@@ -4557,7 +4547,7 @@
         <v>57</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>769</v>
+        <v>767</v>
       </c>
       <c r="F11" s="25" t="s">
         <v>289</v>
@@ -4569,7 +4559,7 @@
         <v>124</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>1034</v>
+        <v>1032</v>
       </c>
       <c r="J11" s="6" t="s">
         <v>628</v>
@@ -4594,7 +4584,7 @@
         <v>57</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="F12" s="25" t="s">
         <v>299</v>
@@ -4603,7 +4593,7 @@
         <v>87</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>996</v>
+        <v>994</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>86</v>
@@ -4631,13 +4621,13 @@
         <v>57</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
       <c r="F13" s="25" t="s">
         <v>301</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>956</v>
+        <v>954</v>
       </c>
       <c r="H13" s="2" t="s">
         <v>75</v>
@@ -4668,7 +4658,7 @@
         <v>47</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>772</v>
+        <v>770</v>
       </c>
       <c r="F14" s="26" t="s">
         <v>319</v>
@@ -4683,7 +4673,7 @@
         <v>655</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>1072</v>
+        <v>1070</v>
       </c>
       <c r="K14" s="5" t="s">
         <v>454</v>
@@ -4702,10 +4692,10 @@
         <v>14</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="F15" s="26" t="s">
         <v>694</v>
@@ -4720,7 +4710,7 @@
         <v>396</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>1073</v>
+        <v>1071</v>
       </c>
       <c r="K15" s="5" t="s">
         <v>454</v>
@@ -4739,10 +4729,10 @@
         <v>14</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>774</v>
+        <v>772</v>
       </c>
       <c r="F16" s="26" t="s">
         <v>692</v>
@@ -4754,7 +4744,7 @@
         <v>387</v>
       </c>
       <c r="I16" s="12" t="s">
-        <v>1035</v>
+        <v>1033</v>
       </c>
       <c r="J16" s="1" t="s">
         <v>389</v>
@@ -4779,13 +4769,13 @@
         <v>1</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>775</v>
+        <v>773</v>
       </c>
       <c r="F17" s="25" t="s">
         <v>253</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>957</v>
+        <v>955</v>
       </c>
       <c r="H17" s="2" t="s">
         <v>226</v>
@@ -4816,13 +4806,13 @@
         <v>1</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="F18" s="25" t="s">
         <v>279</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>958</v>
+        <v>956</v>
       </c>
       <c r="H18" s="2" t="s">
         <v>151</v>
@@ -4853,7 +4843,7 @@
         <v>1</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="F19" s="25" t="s">
         <v>282</v>
@@ -4862,7 +4852,7 @@
         <v>139</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>997</v>
+        <v>995</v>
       </c>
       <c r="I19" s="2" t="s">
         <v>138</v>
@@ -4890,10 +4880,10 @@
         <v>1</v>
       </c>
       <c r="E20" s="37" t="s">
-        <v>778</v>
+        <v>776</v>
       </c>
       <c r="F20" s="31" t="s">
-        <v>1132</v>
+        <v>1130</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>441</v>
@@ -4927,7 +4917,7 @@
         <v>1</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>779</v>
+        <v>777</v>
       </c>
       <c r="F21" s="25" t="s">
         <v>283</v>
@@ -4936,7 +4926,7 @@
         <v>135</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>998</v>
+        <v>996</v>
       </c>
       <c r="I21" s="2" t="s">
         <v>134</v>
@@ -4964,13 +4954,13 @@
         <v>1</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>780</v>
+        <v>778</v>
       </c>
       <c r="F22" s="25" t="s">
         <v>320</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>959</v>
+        <v>957</v>
       </c>
       <c r="H22" s="2" t="s">
         <v>102</v>
@@ -5001,7 +4991,7 @@
         <v>1</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>781</v>
+        <v>779</v>
       </c>
       <c r="F23" s="26" t="s">
         <v>576</v>
@@ -5010,7 +5000,7 @@
         <v>498</v>
       </c>
       <c r="H23" s="12" t="s">
-        <v>999</v>
+        <v>997</v>
       </c>
       <c r="I23" s="12" t="s">
         <v>499</v>
@@ -5038,7 +5028,7 @@
         <v>1</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>782</v>
+        <v>780</v>
       </c>
       <c r="F24" s="26" t="s">
         <v>584</v>
@@ -5050,7 +5040,7 @@
         <v>585</v>
       </c>
       <c r="I24" s="12" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J24" s="1" t="s">
         <v>535</v>
@@ -5075,7 +5065,7 @@
         <v>81</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="F25" s="25" t="s">
         <v>683</v>
@@ -5087,7 +5077,7 @@
         <v>80</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
       <c r="J25" s="6" t="s">
         <v>645</v>
@@ -5111,7 +5101,7 @@
         <v>28</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
       <c r="F26" s="26" t="s">
         <v>688</v>
@@ -5123,7 +5113,7 @@
         <v>27</v>
       </c>
       <c r="I26" s="12" t="s">
-        <v>1038</v>
+        <v>1036</v>
       </c>
       <c r="J26" s="1" t="s">
         <v>660</v>
@@ -5148,13 +5138,13 @@
         <v>5</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>785</v>
+        <v>783</v>
       </c>
       <c r="F27" s="26" t="s">
         <v>315</v>
       </c>
       <c r="G27" s="12" t="s">
-        <v>960</v>
+        <v>958</v>
       </c>
       <c r="H27" s="12" t="s">
         <v>4</v>
@@ -5185,7 +5175,7 @@
         <v>183</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>786</v>
+        <v>784</v>
       </c>
       <c r="F28" s="25" t="s">
         <v>268</v>
@@ -5197,7 +5187,7 @@
         <v>182</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>1039</v>
+        <v>1037</v>
       </c>
       <c r="J28" s="6" t="s">
         <v>340</v>
@@ -5219,10 +5209,10 @@
         <v>14</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>787</v>
+        <v>785</v>
       </c>
       <c r="F29" s="26" t="s">
         <v>695</v>
@@ -5234,7 +5224,7 @@
         <v>406</v>
       </c>
       <c r="I29" s="12" t="s">
-        <v>1040</v>
+        <v>1038</v>
       </c>
       <c r="J29" s="1" t="s">
         <v>408</v>
@@ -5259,7 +5249,7 @@
         <v>1</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>788</v>
+        <v>786</v>
       </c>
       <c r="F30" s="26" t="s">
         <v>573</v>
@@ -5268,7 +5258,7 @@
         <v>493</v>
       </c>
       <c r="H30" s="12" t="s">
-        <v>1000</v>
+        <v>998</v>
       </c>
       <c r="I30" s="12" t="s">
         <v>494</v>
@@ -5293,16 +5283,16 @@
         <v>14</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>789</v>
+        <v>787</v>
       </c>
       <c r="F31" s="26" t="s">
         <v>573</v>
       </c>
       <c r="G31" s="12" t="s">
-        <v>961</v>
+        <v>959</v>
       </c>
       <c r="H31" s="12" t="s">
         <v>134</v>
@@ -5330,16 +5320,16 @@
         <v>14</v>
       </c>
       <c r="D32" s="11" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>790</v>
+        <v>788</v>
       </c>
       <c r="F32" s="26" t="s">
         <v>563</v>
       </c>
       <c r="G32" s="12" t="s">
-        <v>962</v>
+        <v>960</v>
       </c>
       <c r="H32" s="12" t="s">
         <v>424</v>
@@ -5367,10 +5357,10 @@
         <v>14</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>791</v>
+        <v>789</v>
       </c>
       <c r="F33" s="26" t="s">
         <v>564</v>
@@ -5382,7 +5372,7 @@
         <v>433</v>
       </c>
       <c r="I33" s="12" t="s">
-        <v>1041</v>
+        <v>1039</v>
       </c>
       <c r="J33" s="1" t="s">
         <v>435</v>
@@ -5404,10 +5394,10 @@
         <v>14</v>
       </c>
       <c r="D34" s="11" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="E34" s="9" t="s">
-        <v>792</v>
+        <v>790</v>
       </c>
       <c r="F34" s="26" t="s">
         <v>565</v>
@@ -5422,7 +5412,7 @@
         <v>438</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>1074</v>
+        <v>1072</v>
       </c>
       <c r="K34" s="5" t="s">
         <v>454</v>
@@ -5441,10 +5431,10 @@
         <v>14</v>
       </c>
       <c r="D35" s="11" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>793</v>
+        <v>791</v>
       </c>
       <c r="F35" s="26" t="s">
         <v>566</v>
@@ -5453,7 +5443,7 @@
         <v>439</v>
       </c>
       <c r="H35" s="12" t="s">
-        <v>1001</v>
+        <v>999</v>
       </c>
       <c r="I35" s="12" t="s">
         <v>440</v>
@@ -5478,10 +5468,10 @@
         <v>14</v>
       </c>
       <c r="D36" s="11" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="E36" s="9" t="s">
-        <v>794</v>
+        <v>792</v>
       </c>
       <c r="F36" s="26" t="s">
         <v>699</v>
@@ -5490,7 +5480,7 @@
         <v>397</v>
       </c>
       <c r="H36" s="12" t="s">
-        <v>1002</v>
+        <v>1000</v>
       </c>
       <c r="I36" s="12" t="s">
         <v>398</v>
@@ -5515,16 +5505,16 @@
         <v>14</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>795</v>
+        <v>793</v>
       </c>
       <c r="F37" s="26" t="s">
         <v>557</v>
       </c>
       <c r="G37" s="12" t="s">
-        <v>963</v>
+        <v>961</v>
       </c>
       <c r="H37" s="12" t="s">
         <v>382</v>
@@ -5555,7 +5545,7 @@
         <v>106</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>796</v>
+        <v>794</v>
       </c>
       <c r="F38" s="26" t="s">
         <v>574</v>
@@ -5567,7 +5557,7 @@
         <v>481</v>
       </c>
       <c r="I38" s="12" t="s">
-        <v>1042</v>
+        <v>1040</v>
       </c>
       <c r="J38" s="1" t="s">
         <v>483</v>
@@ -5592,7 +5582,7 @@
         <v>57</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>797</v>
+        <v>795</v>
       </c>
       <c r="F39" s="26" t="s">
         <v>571</v>
@@ -5604,7 +5594,7 @@
         <v>478</v>
       </c>
       <c r="I39" s="12" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
       <c r="J39" s="1" t="s">
         <v>480</v>
@@ -5629,7 +5619,7 @@
         <v>43</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>798</v>
+        <v>796</v>
       </c>
       <c r="F40" s="26" t="s">
         <v>575</v>
@@ -5663,10 +5653,10 @@
         <v>14</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>799</v>
+        <v>797</v>
       </c>
       <c r="F41" s="26" t="s">
         <v>701</v>
@@ -5678,7 +5668,7 @@
         <v>442</v>
       </c>
       <c r="I41" s="12" t="s">
-        <v>1044</v>
+        <v>1042</v>
       </c>
       <c r="J41" s="1" t="s">
         <v>444</v>
@@ -5700,13 +5690,13 @@
         <v>14</v>
       </c>
       <c r="D42" s="11" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="E42" s="9" t="s">
-        <v>800</v>
+        <v>798</v>
       </c>
       <c r="F42" s="26" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="G42" s="12" t="s">
         <v>24</v>
@@ -5737,10 +5727,10 @@
         <v>14</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>801</v>
+        <v>799</v>
       </c>
       <c r="F43" s="26" t="s">
         <v>691</v>
@@ -5749,7 +5739,7 @@
         <v>384</v>
       </c>
       <c r="H43" s="12" t="s">
-        <v>1003</v>
+        <v>1001</v>
       </c>
       <c r="I43" s="12" t="s">
         <v>385</v>
@@ -5774,10 +5764,10 @@
         <v>14</v>
       </c>
       <c r="D44" s="11" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="E44" s="9" t="s">
-        <v>802</v>
+        <v>800</v>
       </c>
       <c r="F44" s="26" t="s">
         <v>568</v>
@@ -5792,7 +5782,7 @@
         <v>450</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>1075</v>
+        <v>1073</v>
       </c>
       <c r="K44" s="5" t="s">
         <v>454</v>
@@ -5811,10 +5801,10 @@
         <v>14</v>
       </c>
       <c r="D45" s="11" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>803</v>
+        <v>801</v>
       </c>
       <c r="F45" s="26" t="s">
         <v>562</v>
@@ -5829,7 +5819,7 @@
         <v>423</v>
       </c>
       <c r="J45" s="1" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="K45" s="5" t="s">
         <v>454</v>
@@ -5848,10 +5838,10 @@
         <v>14</v>
       </c>
       <c r="D46" s="11" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="E46" s="9" t="s">
-        <v>804</v>
+        <v>802</v>
       </c>
       <c r="F46" s="26" t="s">
         <v>567</v>
@@ -5860,7 +5850,7 @@
         <v>445</v>
       </c>
       <c r="H46" s="12" t="s">
-        <v>1004</v>
+        <v>1002</v>
       </c>
       <c r="I46" s="12" t="s">
         <v>446</v>
@@ -5885,10 +5875,10 @@
         <v>14</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="E47" s="9" t="s">
-        <v>805</v>
+        <v>803</v>
       </c>
       <c r="F47" s="26" t="s">
         <v>561</v>
@@ -5900,7 +5890,7 @@
         <v>418</v>
       </c>
       <c r="I47" s="12" t="s">
-        <v>1045</v>
+        <v>1043</v>
       </c>
       <c r="J47" s="1" t="s">
         <v>420</v>
@@ -5922,16 +5912,16 @@
         <v>14</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="E48" s="9" t="s">
-        <v>806</v>
+        <v>804</v>
       </c>
       <c r="F48" s="26" t="s">
         <v>560</v>
       </c>
       <c r="G48" s="12" t="s">
-        <v>964</v>
+        <v>962</v>
       </c>
       <c r="H48" s="12" t="s">
         <v>409</v>
@@ -5959,10 +5949,10 @@
         <v>14</v>
       </c>
       <c r="D49" s="11" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="E49" s="9" t="s">
-        <v>807</v>
+        <v>805</v>
       </c>
       <c r="F49" s="26" t="s">
         <v>702</v>
@@ -5971,7 +5961,7 @@
         <v>459</v>
       </c>
       <c r="H49" s="12" t="s">
-        <v>1005</v>
+        <v>1003</v>
       </c>
       <c r="I49" s="12" t="s">
         <v>460</v>
@@ -5996,13 +5986,13 @@
         <v>14</v>
       </c>
       <c r="D50" s="11" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="E50" s="37" t="s">
-        <v>808</v>
+        <v>806</v>
       </c>
       <c r="F50" s="32" t="s">
-        <v>1133</v>
+        <v>1131</v>
       </c>
       <c r="G50" s="12" t="s">
         <v>427</v>
@@ -6014,7 +6004,7 @@
         <v>429</v>
       </c>
       <c r="J50" s="33" t="s">
-        <v>1134</v>
+        <v>1132</v>
       </c>
       <c r="K50" s="5" t="s">
         <v>454</v>
@@ -6033,10 +6023,10 @@
         <v>14</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="E51" s="9" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="F51" s="26" t="s">
         <v>558</v>
@@ -6051,7 +6041,7 @@
         <v>402</v>
       </c>
       <c r="J51" s="1" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
       <c r="K51" s="5" t="s">
         <v>454</v>
@@ -6070,13 +6060,13 @@
         <v>14</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="E52" s="9" t="s">
-        <v>810</v>
+        <v>808</v>
       </c>
       <c r="F52" s="26" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="G52" s="12" t="s">
         <v>468</v>
@@ -6088,7 +6078,7 @@
         <v>470</v>
       </c>
       <c r="J52" s="1" t="s">
-        <v>1078</v>
+        <v>1076</v>
       </c>
       <c r="K52" s="5" t="s">
         <v>454</v>
@@ -6107,10 +6097,10 @@
         <v>14</v>
       </c>
       <c r="D53" s="11" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="E53" s="9" t="s">
-        <v>811</v>
+        <v>809</v>
       </c>
       <c r="F53" s="26" t="s">
         <v>703</v>
@@ -6125,7 +6115,7 @@
         <v>464</v>
       </c>
       <c r="J53" s="1" t="s">
-        <v>1079</v>
+        <v>1077</v>
       </c>
       <c r="K53" s="5" t="s">
         <v>454</v>
@@ -6147,7 +6137,7 @@
         <v>19</v>
       </c>
       <c r="E54" s="9" t="s">
-        <v>812</v>
+        <v>810</v>
       </c>
       <c r="F54" s="25" t="s">
         <v>248</v>
@@ -6162,7 +6152,7 @@
         <v>589</v>
       </c>
       <c r="J54" s="6" t="s">
-        <v>1080</v>
+        <v>1078</v>
       </c>
       <c r="K54" s="5" t="s">
         <v>454</v>
@@ -6184,7 +6174,7 @@
         <v>19</v>
       </c>
       <c r="E55" s="9" t="s">
-        <v>813</v>
+        <v>811</v>
       </c>
       <c r="F55" s="25" t="s">
         <v>260</v>
@@ -6221,10 +6211,10 @@
         <v>19</v>
       </c>
       <c r="E56" s="37" t="s">
-        <v>814</v>
+        <v>812</v>
       </c>
       <c r="F56" s="31" t="s">
-        <v>1135</v>
+        <v>1133</v>
       </c>
       <c r="G56" s="2" t="s">
         <v>201</v>
@@ -6258,7 +6248,7 @@
         <v>19</v>
       </c>
       <c r="E57" s="9" t="s">
-        <v>815</v>
+        <v>813</v>
       </c>
       <c r="F57" s="25" t="s">
         <v>263</v>
@@ -6267,7 +6257,7 @@
         <v>196</v>
       </c>
       <c r="H57" s="2" t="s">
-        <v>1006</v>
+        <v>1004</v>
       </c>
       <c r="I57" s="2" t="s">
         <v>195</v>
@@ -6295,7 +6285,7 @@
         <v>19</v>
       </c>
       <c r="E58" s="9" t="s">
-        <v>816</v>
+        <v>814</v>
       </c>
       <c r="F58" s="25" t="s">
         <v>549</v>
@@ -6310,7 +6300,7 @@
         <v>609</v>
       </c>
       <c r="J58" s="6" t="s">
-        <v>1081</v>
+        <v>1079</v>
       </c>
       <c r="K58" s="5" t="s">
         <v>454</v>
@@ -6332,7 +6322,7 @@
         <v>19</v>
       </c>
       <c r="E59" s="9" t="s">
-        <v>817</v>
+        <v>815</v>
       </c>
       <c r="F59" s="25" t="s">
         <v>270</v>
@@ -6344,7 +6334,7 @@
         <v>172</v>
       </c>
       <c r="I59" s="2" t="s">
-        <v>1046</v>
+        <v>1044</v>
       </c>
       <c r="J59" s="6" t="s">
         <v>596</v>
@@ -6369,13 +6359,13 @@
         <v>19</v>
       </c>
       <c r="E60" s="9" t="s">
-        <v>818</v>
+        <v>816</v>
       </c>
       <c r="F60" s="25" t="s">
         <v>614</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>965</v>
+        <v>963</v>
       </c>
       <c r="H60" s="2" t="s">
         <v>161</v>
@@ -6406,7 +6396,7 @@
         <v>19</v>
       </c>
       <c r="E61" s="9" t="s">
-        <v>819</v>
+        <v>817</v>
       </c>
       <c r="F61" s="25" t="s">
         <v>277</v>
@@ -6443,13 +6433,13 @@
         <v>19</v>
       </c>
       <c r="E62" s="9" t="s">
-        <v>820</v>
+        <v>818</v>
       </c>
       <c r="F62" s="25" t="s">
         <v>678</v>
       </c>
       <c r="G62" s="2" t="s">
-        <v>966</v>
+        <v>964</v>
       </c>
       <c r="H62" s="2" t="s">
         <v>156</v>
@@ -6480,7 +6470,7 @@
         <v>19</v>
       </c>
       <c r="E63" s="9" t="s">
-        <v>821</v>
+        <v>819</v>
       </c>
       <c r="F63" s="25" t="s">
         <v>679</v>
@@ -6517,7 +6507,7 @@
         <v>19</v>
       </c>
       <c r="E64" s="9" t="s">
-        <v>822</v>
+        <v>820</v>
       </c>
       <c r="F64" s="25" t="s">
         <v>288</v>
@@ -6526,7 +6516,7 @@
         <v>126</v>
       </c>
       <c r="H64" s="2" t="s">
-        <v>1007</v>
+        <v>1005</v>
       </c>
       <c r="I64" s="2" t="s">
         <v>125</v>
@@ -6554,7 +6544,7 @@
         <v>19</v>
       </c>
       <c r="E65" s="9" t="s">
-        <v>823</v>
+        <v>821</v>
       </c>
       <c r="F65" s="25" t="s">
         <v>294</v>
@@ -6566,7 +6556,7 @@
         <v>111</v>
       </c>
       <c r="I65" s="2" t="s">
-        <v>1047</v>
+        <v>1045</v>
       </c>
       <c r="J65" s="6" t="s">
         <v>0</v>
@@ -6591,7 +6581,7 @@
         <v>19</v>
       </c>
       <c r="E66" s="9" t="s">
-        <v>824</v>
+        <v>822</v>
       </c>
       <c r="F66" s="25" t="s">
         <v>550</v>
@@ -6628,10 +6618,10 @@
         <v>19</v>
       </c>
       <c r="E67" s="37" t="s">
-        <v>825</v>
+        <v>823</v>
       </c>
       <c r="F67" s="31" t="s">
-        <v>1136</v>
+        <v>1134</v>
       </c>
       <c r="G67" s="2" t="s">
         <v>21</v>
@@ -6665,7 +6655,7 @@
         <v>19</v>
       </c>
       <c r="E68" s="9" t="s">
-        <v>826</v>
+        <v>824</v>
       </c>
       <c r="F68" s="25" t="s">
         <v>551</v>
@@ -6702,7 +6692,7 @@
         <v>19</v>
       </c>
       <c r="E69" s="9" t="s">
-        <v>827</v>
+        <v>825</v>
       </c>
       <c r="F69" s="25" t="s">
         <v>552</v>
@@ -6739,10 +6729,10 @@
         <v>19</v>
       </c>
       <c r="E70" s="9" t="s">
-        <v>828</v>
+        <v>826</v>
       </c>
       <c r="F70" s="26" t="s">
-        <v>1109</v>
+        <v>1107</v>
       </c>
       <c r="G70" s="12" t="s">
         <v>24</v>
@@ -6776,10 +6766,10 @@
         <v>19</v>
       </c>
       <c r="E71" s="9" t="s">
-        <v>829</v>
+        <v>827</v>
       </c>
       <c r="F71" s="26" t="s">
-        <v>1110</v>
+        <v>1108</v>
       </c>
       <c r="G71" s="12" t="s">
         <v>21</v>
@@ -6813,7 +6803,7 @@
         <v>45</v>
       </c>
       <c r="E72" s="9" t="s">
-        <v>830</v>
+        <v>828</v>
       </c>
       <c r="F72" s="26" t="s">
         <v>307</v>
@@ -6850,7 +6840,7 @@
         <v>113</v>
       </c>
       <c r="E73" s="9" t="s">
-        <v>831</v>
+        <v>829</v>
       </c>
       <c r="F73" s="25" t="s">
         <v>265</v>
@@ -6865,7 +6855,7 @@
         <v>606</v>
       </c>
       <c r="J73" s="6" t="s">
-        <v>1082</v>
+        <v>1080</v>
       </c>
       <c r="K73" s="5" t="s">
         <v>454</v>
@@ -6887,13 +6877,13 @@
         <v>113</v>
       </c>
       <c r="E74" s="9" t="s">
-        <v>832</v>
+        <v>830</v>
       </c>
       <c r="F74" s="25" t="s">
         <v>281</v>
       </c>
       <c r="G74" s="2" t="s">
-        <v>967</v>
+        <v>965</v>
       </c>
       <c r="H74" s="2" t="s">
         <v>141</v>
@@ -6924,19 +6914,19 @@
         <v>113</v>
       </c>
       <c r="E75" s="37" t="s">
-        <v>833</v>
+        <v>831</v>
       </c>
       <c r="F75" s="25" t="s">
         <v>293</v>
       </c>
       <c r="G75" s="2" t="s">
-        <v>968</v>
+        <v>966</v>
       </c>
       <c r="H75" s="2" t="s">
         <v>112</v>
       </c>
       <c r="I75" s="34" t="s">
-        <v>1137</v>
+        <v>1135</v>
       </c>
       <c r="J75" s="6" t="s">
         <v>632</v>
@@ -6961,13 +6951,13 @@
         <v>11</v>
       </c>
       <c r="E76" s="9" t="s">
-        <v>834</v>
+        <v>832</v>
       </c>
       <c r="F76" s="26" t="s">
         <v>537</v>
       </c>
       <c r="G76" s="12" t="s">
-        <v>969</v>
+        <v>967</v>
       </c>
       <c r="H76" s="12" t="s">
         <v>323</v>
@@ -6997,7 +6987,7 @@
         <v>11</v>
       </c>
       <c r="E77" s="9" t="s">
-        <v>835</v>
+        <v>833</v>
       </c>
       <c r="F77" s="26" t="s">
         <v>690</v>
@@ -7006,7 +6996,7 @@
         <v>332</v>
       </c>
       <c r="H77" s="12" t="s">
-        <v>1008</v>
+        <v>1006</v>
       </c>
       <c r="I77" s="12" t="s">
         <v>333</v>
@@ -7034,7 +7024,7 @@
         <v>57</v>
       </c>
       <c r="E78" s="9" t="s">
-        <v>836</v>
+        <v>834</v>
       </c>
       <c r="F78" s="26" t="s">
         <v>536</v>
@@ -7043,7 +7033,7 @@
         <v>206</v>
       </c>
       <c r="H78" s="12" t="s">
-        <v>1009</v>
+        <v>1007</v>
       </c>
       <c r="I78" s="12" t="s">
         <v>321</v>
@@ -7071,7 +7061,7 @@
         <v>31</v>
       </c>
       <c r="E79" s="9" t="s">
-        <v>837</v>
+        <v>835</v>
       </c>
       <c r="F79" s="26" t="s">
         <v>311</v>
@@ -7108,10 +7098,10 @@
         <v>31</v>
       </c>
       <c r="E80" s="37" t="s">
-        <v>838</v>
+        <v>836</v>
       </c>
       <c r="F80" s="32" t="s">
-        <v>1138</v>
+        <v>1136</v>
       </c>
       <c r="G80" s="12" t="s">
         <v>30</v>
@@ -7145,7 +7135,7 @@
         <v>31</v>
       </c>
       <c r="E81" s="9" t="s">
-        <v>839</v>
+        <v>837</v>
       </c>
       <c r="F81" s="26" t="s">
         <v>538</v>
@@ -7160,7 +7150,7 @@
         <v>328</v>
       </c>
       <c r="J81" s="1" t="s">
-        <v>1083</v>
+        <v>1081</v>
       </c>
       <c r="K81" s="5" t="s">
         <v>454</v>
@@ -7182,7 +7172,7 @@
         <v>46</v>
       </c>
       <c r="E82" s="9" t="s">
-        <v>840</v>
+        <v>838</v>
       </c>
       <c r="F82" s="26" t="s">
         <v>544</v>
@@ -7194,7 +7184,7 @@
         <v>350</v>
       </c>
       <c r="I82" s="12" t="s">
-        <v>1048</v>
+        <v>1046</v>
       </c>
       <c r="J82" s="1" t="s">
         <v>352</v>
@@ -7219,7 +7209,7 @@
         <v>66</v>
       </c>
       <c r="E83" s="9" t="s">
-        <v>841</v>
+        <v>839</v>
       </c>
       <c r="F83" s="25" t="s">
         <v>667</v>
@@ -7231,7 +7221,7 @@
         <v>242</v>
       </c>
       <c r="I83" s="2" t="s">
-        <v>1049</v>
+        <v>1047</v>
       </c>
       <c r="J83" s="6" t="s">
         <v>466</v>
@@ -7256,7 +7246,7 @@
         <v>66</v>
       </c>
       <c r="E84" s="9" t="s">
-        <v>842</v>
+        <v>840</v>
       </c>
       <c r="F84" s="25" t="s">
         <v>246</v>
@@ -7268,7 +7258,7 @@
         <v>233</v>
       </c>
       <c r="I84" s="2" t="s">
-        <v>1050</v>
+        <v>1048</v>
       </c>
       <c r="J84" s="6" t="s">
         <v>2</v>
@@ -7293,13 +7283,13 @@
         <v>66</v>
       </c>
       <c r="E85" s="9" t="s">
-        <v>843</v>
+        <v>841</v>
       </c>
       <c r="F85" s="25" t="s">
         <v>254</v>
       </c>
       <c r="G85" s="2" t="s">
-        <v>953</v>
+        <v>951</v>
       </c>
       <c r="H85" s="2" t="s">
         <v>224</v>
@@ -7330,13 +7320,13 @@
         <v>66</v>
       </c>
       <c r="E86" s="9" t="s">
-        <v>844</v>
+        <v>842</v>
       </c>
       <c r="F86" s="25" t="s">
         <v>266</v>
       </c>
       <c r="G86" s="2" t="s">
-        <v>970</v>
+        <v>968</v>
       </c>
       <c r="H86" s="2" t="s">
         <v>187</v>
@@ -7367,7 +7357,7 @@
         <v>66</v>
       </c>
       <c r="E87" s="9" t="s">
-        <v>845</v>
+        <v>843</v>
       </c>
       <c r="F87" s="25" t="s">
         <v>682</v>
@@ -7379,7 +7369,7 @@
         <v>93</v>
       </c>
       <c r="I87" s="2" t="s">
-        <v>969</v>
+        <v>967</v>
       </c>
       <c r="J87" s="6" t="s">
         <v>638</v>
@@ -7404,7 +7394,7 @@
         <v>66</v>
       </c>
       <c r="E88" s="9" t="s">
-        <v>846</v>
+        <v>844</v>
       </c>
       <c r="F88" s="25" t="s">
         <v>641</v>
@@ -7440,7 +7430,7 @@
         <v>66</v>
       </c>
       <c r="E89" s="9" t="s">
-        <v>847</v>
+        <v>845</v>
       </c>
       <c r="F89" s="25" t="s">
         <v>643</v>
@@ -7452,7 +7442,7 @@
         <v>85</v>
       </c>
       <c r="I89" s="2" t="s">
-        <v>1051</v>
+        <v>1049</v>
       </c>
       <c r="J89" s="6" t="s">
         <v>644</v>
@@ -7477,13 +7467,13 @@
         <v>66</v>
       </c>
       <c r="E90" s="37" t="s">
-        <v>848</v>
+        <v>846</v>
       </c>
       <c r="F90" s="31" t="s">
-        <v>1139</v>
+        <v>1137</v>
       </c>
       <c r="G90" s="2" t="s">
-        <v>971</v>
+        <v>969</v>
       </c>
       <c r="H90" s="2" t="s">
         <v>64</v>
@@ -7513,7 +7503,7 @@
         <v>58</v>
       </c>
       <c r="E91" s="9" t="s">
-        <v>849</v>
+        <v>847</v>
       </c>
       <c r="F91" s="25" t="s">
         <v>255</v>
@@ -7528,7 +7518,7 @@
         <v>592</v>
       </c>
       <c r="J91" s="6" t="s">
-        <v>1084</v>
+        <v>1082</v>
       </c>
       <c r="K91" s="5" t="s">
         <v>454</v>
@@ -7550,7 +7540,7 @@
         <v>58</v>
       </c>
       <c r="E92" s="9" t="s">
-        <v>850</v>
+        <v>848</v>
       </c>
       <c r="F92" s="25" t="s">
         <v>261</v>
@@ -7562,7 +7552,7 @@
         <v>199</v>
       </c>
       <c r="I92" s="6" t="s">
-        <v>1085</v>
+        <v>1083</v>
       </c>
       <c r="J92" s="2" t="s">
         <v>2</v>
@@ -7586,7 +7576,7 @@
         <v>58</v>
       </c>
       <c r="E93" s="9" t="s">
-        <v>851</v>
+        <v>849</v>
       </c>
       <c r="F93" s="25" t="s">
         <v>264</v>
@@ -7620,10 +7610,10 @@
         <v>14</v>
       </c>
       <c r="D94" s="11" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="E94" s="9" t="s">
-        <v>852</v>
+        <v>850</v>
       </c>
       <c r="F94" s="26" t="s">
         <v>540</v>
@@ -7656,16 +7646,16 @@
         <v>14</v>
       </c>
       <c r="D95" s="11" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="E95" s="9" t="s">
-        <v>853</v>
+        <v>851</v>
       </c>
       <c r="F95" s="26" t="s">
         <v>548</v>
       </c>
       <c r="G95" s="12" t="s">
-        <v>972</v>
+        <v>970</v>
       </c>
       <c r="H95" s="12" t="s">
         <v>363</v>
@@ -7696,7 +7686,7 @@
         <v>71</v>
       </c>
       <c r="E96" s="9" t="s">
-        <v>854</v>
+        <v>852</v>
       </c>
       <c r="F96" s="25" t="s">
         <v>302</v>
@@ -7705,7 +7695,7 @@
         <v>70</v>
       </c>
       <c r="H96" s="2" t="s">
-        <v>1010</v>
+        <v>1008</v>
       </c>
       <c r="I96" s="2" t="s">
         <v>69</v>
@@ -7733,7 +7723,7 @@
         <v>68</v>
       </c>
       <c r="E97" s="37" t="s">
-        <v>855</v>
+        <v>853</v>
       </c>
       <c r="F97" s="25" t="s">
         <v>284</v>
@@ -7745,7 +7735,7 @@
         <v>132</v>
       </c>
       <c r="I97" s="35" t="s">
-        <v>1087</v>
+        <v>1085</v>
       </c>
       <c r="J97" s="36" t="s">
         <v>0</v>
@@ -7770,7 +7760,7 @@
         <v>68</v>
       </c>
       <c r="E98" s="9" t="s">
-        <v>856</v>
+        <v>854</v>
       </c>
       <c r="F98" s="25" t="s">
         <v>303</v>
@@ -7782,7 +7772,7 @@
         <v>67</v>
       </c>
       <c r="I98" s="2" t="s">
-        <v>1052</v>
+        <v>1050</v>
       </c>
       <c r="J98" s="6" t="s">
         <v>651</v>
@@ -7807,7 +7797,7 @@
         <v>33</v>
       </c>
       <c r="E99" s="9" t="s">
-        <v>857</v>
+        <v>855</v>
       </c>
       <c r="F99" s="26" t="s">
         <v>577</v>
@@ -7822,7 +7812,7 @@
         <v>503</v>
       </c>
       <c r="J99" s="1" t="s">
-        <v>1088</v>
+        <v>1086</v>
       </c>
       <c r="K99" s="5" t="s">
         <v>454</v>
@@ -7844,7 +7834,7 @@
         <v>33</v>
       </c>
       <c r="E100" s="9" t="s">
-        <v>858</v>
+        <v>856</v>
       </c>
       <c r="F100" s="26" t="s">
         <v>579</v>
@@ -7853,7 +7843,7 @@
         <v>504</v>
       </c>
       <c r="H100" s="12" t="s">
-        <v>1011</v>
+        <v>1009</v>
       </c>
       <c r="I100" s="12" t="s">
         <v>505</v>
@@ -7881,7 +7871,7 @@
         <v>33</v>
       </c>
       <c r="E101" s="9" t="s">
-        <v>859</v>
+        <v>857</v>
       </c>
       <c r="F101" s="26" t="s">
         <v>578</v>
@@ -7893,7 +7883,7 @@
         <v>507</v>
       </c>
       <c r="I101" s="12" t="s">
-        <v>1053</v>
+        <v>1051</v>
       </c>
       <c r="J101" s="1" t="s">
         <v>509</v>
@@ -7918,10 +7908,10 @@
         <v>33</v>
       </c>
       <c r="E102" s="9" t="s">
-        <v>860</v>
+        <v>858</v>
       </c>
       <c r="F102" s="26" t="s">
-        <v>1113</v>
+        <v>1111</v>
       </c>
       <c r="G102" s="12" t="s">
         <v>510</v>
@@ -7933,7 +7923,7 @@
         <v>512</v>
       </c>
       <c r="J102" s="1" t="s">
-        <v>1089</v>
+        <v>1087</v>
       </c>
       <c r="K102" s="5" t="s">
         <v>454</v>
@@ -7955,13 +7945,13 @@
         <v>33</v>
       </c>
       <c r="E103" s="9" t="s">
-        <v>861</v>
+        <v>859</v>
       </c>
       <c r="F103" s="26" t="s">
-        <v>1115</v>
+        <v>1113</v>
       </c>
       <c r="G103" s="12" t="s">
-        <v>974</v>
+        <v>972</v>
       </c>
       <c r="H103" s="12" t="s">
         <v>513</v>
@@ -7992,16 +7982,16 @@
         <v>33</v>
       </c>
       <c r="E104" s="9" t="s">
-        <v>862</v>
+        <v>860</v>
       </c>
       <c r="F104" s="26" t="s">
-        <v>1114</v>
+        <v>1112</v>
       </c>
       <c r="G104" s="12" t="s">
         <v>516</v>
       </c>
       <c r="H104" s="12" t="s">
-        <v>1012</v>
+        <v>1010</v>
       </c>
       <c r="I104" s="12" t="s">
         <v>517</v>
@@ -8029,7 +8019,7 @@
         <v>33</v>
       </c>
       <c r="E105" s="9" t="s">
-        <v>863</v>
+        <v>861</v>
       </c>
       <c r="F105" s="26" t="s">
         <v>580</v>
@@ -8041,7 +8031,7 @@
         <v>518</v>
       </c>
       <c r="I105" s="12" t="s">
-        <v>1054</v>
+        <v>1052</v>
       </c>
       <c r="J105" s="1" t="s">
         <v>520</v>
@@ -8066,7 +8056,7 @@
         <v>33</v>
       </c>
       <c r="E106" s="9" t="s">
-        <v>864</v>
+        <v>862</v>
       </c>
       <c r="F106" s="26" t="s">
         <v>581</v>
@@ -8081,7 +8071,7 @@
         <v>523</v>
       </c>
       <c r="J106" s="1" t="s">
-        <v>1090</v>
+        <v>1088</v>
       </c>
       <c r="K106" s="5" t="s">
         <v>454</v>
@@ -8103,13 +8093,13 @@
         <v>33</v>
       </c>
       <c r="E107" s="9" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
       <c r="F107" s="26" t="s">
         <v>582</v>
       </c>
       <c r="G107" s="12" t="s">
-        <v>975</v>
+        <v>973</v>
       </c>
       <c r="H107" s="12" t="s">
         <v>524</v>
@@ -8140,13 +8130,13 @@
         <v>33</v>
       </c>
       <c r="E108" s="9" t="s">
-        <v>866</v>
+        <v>864</v>
       </c>
       <c r="F108" s="26" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="G108" s="12" t="s">
-        <v>976</v>
+        <v>974</v>
       </c>
       <c r="H108" s="12" t="s">
         <v>89</v>
@@ -8177,7 +8167,7 @@
         <v>33</v>
       </c>
       <c r="E109" s="9" t="s">
-        <v>867</v>
+        <v>865</v>
       </c>
       <c r="F109" s="26" t="s">
         <v>583</v>
@@ -8186,7 +8176,7 @@
         <v>528</v>
       </c>
       <c r="H109" s="12" t="s">
-        <v>1013</v>
+        <v>1011</v>
       </c>
       <c r="I109" s="12" t="s">
         <v>529</v>
@@ -8214,7 +8204,7 @@
         <v>33</v>
       </c>
       <c r="E110" s="9" t="s">
-        <v>868</v>
+        <v>866</v>
       </c>
       <c r="F110" s="26" t="s">
         <v>704</v>
@@ -8226,7 +8216,7 @@
         <v>531</v>
       </c>
       <c r="I110" s="12" t="s">
-        <v>1055</v>
+        <v>1053</v>
       </c>
       <c r="J110" s="1" t="s">
         <v>533</v>
@@ -8251,7 +8241,7 @@
         <v>11</v>
       </c>
       <c r="E111" s="9" t="s">
-        <v>869</v>
+        <v>867</v>
       </c>
       <c r="F111" s="25" t="s">
         <v>669</v>
@@ -8260,7 +8250,7 @@
         <v>238</v>
       </c>
       <c r="H111" s="2" t="s">
-        <v>1014</v>
+        <v>1012</v>
       </c>
       <c r="I111" s="2" t="s">
         <v>237</v>
@@ -8288,13 +8278,13 @@
         <v>11</v>
       </c>
       <c r="E112" s="9" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
       <c r="F112" s="32" t="s">
-        <v>1140</v>
+        <v>1138</v>
       </c>
       <c r="G112" s="12" t="s">
-        <v>977</v>
+        <v>975</v>
       </c>
       <c r="H112" s="12" t="s">
         <v>354</v>
@@ -8325,7 +8315,7 @@
         <v>33</v>
       </c>
       <c r="E113" s="9" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
       <c r="F113" s="26" t="s">
         <v>570</v>
@@ -8340,7 +8330,7 @@
         <v>477</v>
       </c>
       <c r="J113" s="12" t="s">
-        <v>1091</v>
+        <v>1089</v>
       </c>
       <c r="K113" s="5" t="s">
         <v>454</v>
@@ -8362,16 +8352,16 @@
         <v>11</v>
       </c>
       <c r="E114" s="37" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
       <c r="F114" s="32" t="s">
-        <v>1141</v>
+        <v>1139</v>
       </c>
       <c r="G114" s="12" t="s">
         <v>484</v>
       </c>
       <c r="H114" s="12" t="s">
-        <v>1015</v>
+        <v>1013</v>
       </c>
       <c r="I114" s="12" t="s">
         <v>485</v>
@@ -8396,19 +8386,19 @@
         <v>14</v>
       </c>
       <c r="D115" s="11" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="E115" s="9" t="s">
-        <v>873</v>
+        <v>871</v>
       </c>
       <c r="F115" s="26" t="s">
-        <v>1117</v>
+        <v>1115</v>
       </c>
       <c r="G115" s="12" t="s">
         <v>545</v>
       </c>
       <c r="H115" s="12" t="s">
-        <v>1016</v>
+        <v>1014</v>
       </c>
       <c r="I115" s="12" t="s">
         <v>361</v>
@@ -8433,19 +8423,19 @@
         <v>14</v>
       </c>
       <c r="D116" s="11" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="E116" s="37" t="s">
-        <v>874</v>
+        <v>872</v>
       </c>
       <c r="F116" s="32" t="s">
-        <v>1142</v>
+        <v>1140</v>
       </c>
       <c r="G116" s="12" t="s">
         <v>430</v>
       </c>
       <c r="H116" s="12" t="s">
-        <v>1017</v>
+        <v>1015</v>
       </c>
       <c r="I116" s="12" t="s">
         <v>431</v>
@@ -8473,10 +8463,10 @@
         <v>19</v>
       </c>
       <c r="E117" s="37" t="s">
-        <v>875</v>
+        <v>873</v>
       </c>
       <c r="F117" s="32" t="s">
-        <v>1143</v>
+        <v>1141</v>
       </c>
       <c r="G117" s="12" t="s">
         <v>23</v>
@@ -8510,10 +8500,10 @@
         <v>82</v>
       </c>
       <c r="E118" s="37" t="s">
-        <v>876</v>
+        <v>874</v>
       </c>
       <c r="F118" s="25" t="s">
-        <v>1130</v>
+        <v>1128</v>
       </c>
       <c r="G118" s="2" t="s">
         <v>146</v>
@@ -8522,10 +8512,10 @@
         <v>147</v>
       </c>
       <c r="I118" s="34" t="s">
-        <v>1145</v>
+        <v>1143</v>
       </c>
       <c r="J118" s="35" t="s">
-        <v>1144</v>
+        <v>1142</v>
       </c>
       <c r="K118" s="5" t="s">
         <v>451</v>
@@ -8547,13 +8537,13 @@
         <v>20</v>
       </c>
       <c r="E119" s="9" t="s">
-        <v>877</v>
+        <v>875</v>
       </c>
       <c r="F119" s="25" t="s">
         <v>245</v>
       </c>
       <c r="G119" s="2" t="s">
-        <v>978</v>
+        <v>976</v>
       </c>
       <c r="H119" s="2" t="s">
         <v>240</v>
@@ -8584,7 +8574,7 @@
         <v>20</v>
       </c>
       <c r="E120" s="9" t="s">
-        <v>878</v>
+        <v>876</v>
       </c>
       <c r="F120" s="25" t="s">
         <v>670</v>
@@ -8596,7 +8586,7 @@
         <v>235</v>
       </c>
       <c r="I120" s="2" t="s">
-        <v>1056</v>
+        <v>1054</v>
       </c>
       <c r="J120" s="6" t="s">
         <v>2</v>
@@ -8621,10 +8611,10 @@
         <v>60</v>
       </c>
       <c r="E121" s="37" t="s">
-        <v>879</v>
+        <v>877</v>
       </c>
       <c r="F121" s="31" t="s">
-        <v>1146</v>
+        <v>1144</v>
       </c>
       <c r="G121" s="2" t="s">
         <v>208</v>
@@ -8657,7 +8647,7 @@
         <v>60</v>
       </c>
       <c r="E122" s="37" t="s">
-        <v>880</v>
+        <v>878</v>
       </c>
       <c r="F122" s="31" t="s">
         <v>290</v>
@@ -8666,7 +8656,7 @@
         <v>122</v>
       </c>
       <c r="H122" s="34" t="s">
-        <v>1147</v>
+        <v>1145</v>
       </c>
       <c r="I122" s="2" t="s">
         <v>121</v>
@@ -8694,10 +8684,10 @@
         <v>60</v>
       </c>
       <c r="E123" s="9" t="s">
-        <v>881</v>
+        <v>879</v>
       </c>
       <c r="F123" s="25" t="s">
-        <v>1118</v>
+        <v>1116</v>
       </c>
       <c r="G123" s="2" t="s">
         <v>119</v>
@@ -8706,7 +8696,7 @@
         <v>120</v>
       </c>
       <c r="I123" s="6" t="s">
-        <v>1057</v>
+        <v>1055</v>
       </c>
       <c r="J123" s="2" t="s">
         <v>630</v>
@@ -8731,7 +8721,7 @@
         <v>28</v>
       </c>
       <c r="E124" s="9" t="s">
-        <v>882</v>
+        <v>880</v>
       </c>
       <c r="F124" s="25" t="s">
         <v>305</v>
@@ -8746,7 +8736,7 @@
         <v>654</v>
       </c>
       <c r="J124" s="6" t="s">
-        <v>1092</v>
+        <v>1090</v>
       </c>
       <c r="K124" s="5" t="s">
         <v>454</v>
@@ -8768,7 +8758,7 @@
         <v>46</v>
       </c>
       <c r="E125" s="9" t="s">
-        <v>883</v>
+        <v>881</v>
       </c>
       <c r="F125" s="25" t="s">
         <v>249</v>
@@ -8780,7 +8770,7 @@
         <v>251</v>
       </c>
       <c r="I125" s="6" t="s">
-        <v>1093</v>
+        <v>1091</v>
       </c>
       <c r="J125" s="2" t="s">
         <v>2</v>
@@ -8803,7 +8793,7 @@
         <v>46</v>
       </c>
       <c r="E126" s="9" t="s">
-        <v>884</v>
+        <v>882</v>
       </c>
       <c r="F126" s="25" t="s">
         <v>258</v>
@@ -8818,7 +8808,7 @@
         <v>595</v>
       </c>
       <c r="J126" s="6" t="s">
-        <v>1094</v>
+        <v>1092</v>
       </c>
       <c r="K126" s="5" t="s">
         <v>454</v>
@@ -8840,7 +8830,7 @@
         <v>46</v>
       </c>
       <c r="E127" s="9" t="s">
-        <v>885</v>
+        <v>883</v>
       </c>
       <c r="F127" s="25" t="s">
         <v>602</v>
@@ -8849,7 +8839,7 @@
         <v>194</v>
       </c>
       <c r="H127" s="2" t="s">
-        <v>1018</v>
+        <v>1016</v>
       </c>
       <c r="I127" s="2" t="s">
         <v>193</v>
@@ -8877,7 +8867,7 @@
         <v>46</v>
       </c>
       <c r="E128" s="37" t="s">
-        <v>886</v>
+        <v>884</v>
       </c>
       <c r="F128" s="25" t="s">
         <v>269</v>
@@ -8889,10 +8879,10 @@
         <v>180</v>
       </c>
       <c r="I128" s="2" t="s">
-        <v>1058</v>
+        <v>1056</v>
       </c>
       <c r="J128" s="35" t="s">
-        <v>1148</v>
+        <v>1146</v>
       </c>
       <c r="K128" s="5" t="s">
         <v>451</v>
@@ -8914,7 +8904,7 @@
         <v>46</v>
       </c>
       <c r="E129" s="9" t="s">
-        <v>887</v>
+        <v>885</v>
       </c>
       <c r="F129" s="25" t="s">
         <v>291</v>
@@ -8923,7 +8913,7 @@
         <v>118</v>
       </c>
       <c r="H129" s="2" t="s">
-        <v>1019</v>
+        <v>1017</v>
       </c>
       <c r="I129" s="2" t="s">
         <v>117</v>
@@ -8951,13 +8941,13 @@
         <v>46</v>
       </c>
       <c r="E130" s="9" t="s">
-        <v>888</v>
+        <v>886</v>
       </c>
       <c r="F130" s="25" t="s">
         <v>648</v>
       </c>
       <c r="G130" s="2" t="s">
-        <v>979</v>
+        <v>977</v>
       </c>
       <c r="H130" s="2" t="s">
         <v>276</v>
@@ -8985,16 +8975,16 @@
         <v>14</v>
       </c>
       <c r="D131" s="11" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="E131" s="9" t="s">
-        <v>889</v>
+        <v>887</v>
       </c>
       <c r="F131" s="26" t="s">
         <v>541</v>
       </c>
       <c r="G131" s="12" t="s">
-        <v>980</v>
+        <v>978</v>
       </c>
       <c r="H131" s="12" t="s">
         <v>338</v>
@@ -9025,19 +9015,19 @@
         <v>61</v>
       </c>
       <c r="E132" s="37" t="s">
-        <v>890</v>
+        <v>888</v>
       </c>
       <c r="F132" s="31" t="s">
+        <v>1147</v>
+      </c>
+      <c r="G132" s="34" t="s">
         <v>1149</v>
       </c>
-      <c r="G132" s="34" t="s">
-        <v>1151</v>
-      </c>
       <c r="H132" s="34" t="s">
-        <v>1152</v>
+        <v>1150</v>
       </c>
       <c r="I132" s="34" t="s">
-        <v>1150</v>
+        <v>1148</v>
       </c>
       <c r="J132" s="35" t="s">
         <v>685</v>
@@ -9059,16 +9049,16 @@
         <v>14</v>
       </c>
       <c r="D133" s="9" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="E133" s="9" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
       <c r="F133" s="25" t="s">
         <v>672</v>
       </c>
       <c r="G133" s="2" t="s">
-        <v>981</v>
+        <v>979</v>
       </c>
       <c r="H133" s="2" t="s">
         <v>220</v>
@@ -9096,10 +9086,10 @@
         <v>14</v>
       </c>
       <c r="D134" s="9" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="E134" s="9" t="s">
-        <v>892</v>
+        <v>890</v>
       </c>
       <c r="F134" s="25" t="s">
         <v>257</v>
@@ -9114,7 +9104,7 @@
         <v>674</v>
       </c>
       <c r="J134" s="6" t="s">
-        <v>1095</v>
+        <v>1093</v>
       </c>
       <c r="K134" s="5" t="s">
         <v>454</v>
@@ -9132,10 +9122,10 @@
         <v>14</v>
       </c>
       <c r="D135" s="9" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="E135" s="9" t="s">
-        <v>893</v>
+        <v>891</v>
       </c>
       <c r="F135" s="25" t="s">
         <v>675</v>
@@ -9147,7 +9137,7 @@
         <v>214</v>
       </c>
       <c r="I135" s="2" t="s">
-        <v>1059</v>
+        <v>1057</v>
       </c>
       <c r="J135" s="6" t="s">
         <v>2</v>
@@ -9169,10 +9159,10 @@
         <v>14</v>
       </c>
       <c r="D136" s="11" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="E136" s="9" t="s">
-        <v>894</v>
+        <v>892</v>
       </c>
       <c r="F136" s="26" t="s">
         <v>693</v>
@@ -9181,7 +9171,7 @@
         <v>390</v>
       </c>
       <c r="H136" s="12" t="s">
-        <v>1020</v>
+        <v>1018</v>
       </c>
       <c r="I136" s="12" t="s">
         <v>177</v>
@@ -9206,13 +9196,13 @@
         <v>14</v>
       </c>
       <c r="D137" s="11" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="E137" s="9" t="s">
-        <v>895</v>
+        <v>893</v>
       </c>
       <c r="F137" s="26" t="s">
-        <v>1119</v>
+        <v>1117</v>
       </c>
       <c r="G137" s="12" t="s">
         <v>366</v>
@@ -9221,7 +9211,7 @@
         <v>365</v>
       </c>
       <c r="I137" s="12" t="s">
-        <v>1060</v>
+        <v>1058</v>
       </c>
       <c r="J137" s="1" t="s">
         <v>367</v>
@@ -9246,13 +9236,13 @@
         <v>1</v>
       </c>
       <c r="E138" s="9" t="s">
-        <v>896</v>
+        <v>894</v>
       </c>
       <c r="F138" s="26" t="s">
-        <v>1131</v>
+        <v>1129</v>
       </c>
       <c r="G138" s="12" t="s">
-        <v>982</v>
+        <v>980</v>
       </c>
       <c r="H138" s="12" t="s">
         <v>18</v>
@@ -9283,7 +9273,7 @@
         <v>78</v>
       </c>
       <c r="E139" s="9" t="s">
-        <v>897</v>
+        <v>895</v>
       </c>
       <c r="F139" s="25" t="s">
         <v>681</v>
@@ -9298,7 +9288,7 @@
         <v>636</v>
       </c>
       <c r="J139" s="6" t="s">
-        <v>1096</v>
+        <v>1094</v>
       </c>
       <c r="K139" s="5" t="s">
         <v>454</v>
@@ -9320,7 +9310,7 @@
         <v>78</v>
       </c>
       <c r="E140" s="9" t="s">
-        <v>898</v>
+        <v>896</v>
       </c>
       <c r="F140" s="25" t="s">
         <v>297</v>
@@ -9329,7 +9319,7 @@
         <v>95</v>
       </c>
       <c r="H140" s="2" t="s">
-        <v>1021</v>
+        <v>1019</v>
       </c>
       <c r="I140" s="2" t="s">
         <v>94</v>
@@ -9357,7 +9347,7 @@
         <v>78</v>
       </c>
       <c r="E141" s="9" t="s">
-        <v>899</v>
+        <v>897</v>
       </c>
       <c r="F141" s="25" t="s">
         <v>298</v>
@@ -9366,7 +9356,7 @@
         <v>91</v>
       </c>
       <c r="H141" s="2" t="s">
-        <v>1022</v>
+        <v>1020</v>
       </c>
       <c r="I141" s="2" t="s">
         <v>90</v>
@@ -9394,7 +9384,7 @@
         <v>78</v>
       </c>
       <c r="E142" s="9" t="s">
-        <v>900</v>
+        <v>898</v>
       </c>
       <c r="F142" s="25" t="s">
         <v>300</v>
@@ -9409,7 +9399,7 @@
         <v>646</v>
       </c>
       <c r="J142" s="6" t="s">
-        <v>1097</v>
+        <v>1095</v>
       </c>
       <c r="K142" s="5" t="s">
         <v>454</v>
@@ -9431,10 +9421,10 @@
         <v>116</v>
       </c>
       <c r="E143" s="9" t="s">
-        <v>901</v>
+        <v>899</v>
       </c>
       <c r="F143" s="25" t="s">
-        <v>1120</v>
+        <v>1118</v>
       </c>
       <c r="G143" s="2" t="s">
         <v>211</v>
@@ -9446,7 +9436,7 @@
         <v>212</v>
       </c>
       <c r="J143" s="6" t="s">
-        <v>1098</v>
+        <v>1096</v>
       </c>
       <c r="K143" s="5" t="s">
         <v>454</v>
@@ -9468,7 +9458,7 @@
         <v>116</v>
       </c>
       <c r="E144" s="9" t="s">
-        <v>902</v>
+        <v>900</v>
       </c>
       <c r="F144" s="25" t="s">
         <v>671</v>
@@ -9477,7 +9467,7 @@
         <v>174</v>
       </c>
       <c r="H144" s="2" t="s">
-        <v>1023</v>
+        <v>1021</v>
       </c>
       <c r="I144" s="2" t="s">
         <v>173</v>
@@ -9505,13 +9495,13 @@
         <v>116</v>
       </c>
       <c r="E145" s="9" t="s">
-        <v>903</v>
+        <v>901</v>
       </c>
       <c r="F145" s="25" t="s">
         <v>271</v>
       </c>
       <c r="G145" s="2" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="H145" s="2" t="s">
         <v>170</v>
@@ -9542,10 +9532,10 @@
         <v>116</v>
       </c>
       <c r="E146" s="9" t="s">
-        <v>904</v>
+        <v>902</v>
       </c>
       <c r="F146" s="25" t="s">
-        <v>1121</v>
+        <v>1119</v>
       </c>
       <c r="G146" s="2" t="s">
         <v>165</v>
@@ -9557,7 +9547,7 @@
         <v>613</v>
       </c>
       <c r="J146" s="6" t="s">
-        <v>1065</v>
+        <v>1063</v>
       </c>
       <c r="K146" s="5" t="s">
         <v>454</v>
@@ -9579,10 +9569,10 @@
         <v>116</v>
       </c>
       <c r="E147" s="37" t="s">
-        <v>905</v>
+        <v>903</v>
       </c>
       <c r="F147" s="25" t="s">
-        <v>1156</v>
+        <v>1154</v>
       </c>
       <c r="G147" s="2" t="s">
         <v>145</v>
@@ -9591,7 +9581,7 @@
         <v>144</v>
       </c>
       <c r="I147" s="34" t="s">
-        <v>1153</v>
+        <v>1151</v>
       </c>
       <c r="J147" s="35" t="s">
         <v>2</v>
@@ -9615,7 +9605,7 @@
         <v>116</v>
       </c>
       <c r="E148" s="9" t="s">
-        <v>906</v>
+        <v>904</v>
       </c>
       <c r="F148" s="25" t="s">
         <v>280</v>
@@ -9630,7 +9620,7 @@
         <v>620</v>
       </c>
       <c r="J148" s="6" t="s">
-        <v>1099</v>
+        <v>1097</v>
       </c>
       <c r="K148" s="5" t="s">
         <v>454</v>
@@ -9652,13 +9642,13 @@
         <v>116</v>
       </c>
       <c r="E149" s="9" t="s">
-        <v>907</v>
+        <v>905</v>
       </c>
       <c r="F149" s="25" t="s">
         <v>285</v>
       </c>
       <c r="G149" s="2" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="H149" s="2" t="s">
         <v>131</v>
@@ -9689,7 +9679,7 @@
         <v>116</v>
       </c>
       <c r="E150" s="37" t="s">
-        <v>908</v>
+        <v>906</v>
       </c>
       <c r="F150" s="25" t="s">
         <v>287</v>
@@ -9698,10 +9688,10 @@
         <v>128</v>
       </c>
       <c r="H150" s="2" t="s">
-        <v>1024</v>
+        <v>1022</v>
       </c>
       <c r="I150" s="34" t="s">
-        <v>1154</v>
+        <v>1152</v>
       </c>
       <c r="J150" s="6" t="s">
         <v>2</v>
@@ -9726,7 +9716,7 @@
         <v>116</v>
       </c>
       <c r="E151" s="9" t="s">
-        <v>909</v>
+        <v>907</v>
       </c>
       <c r="F151" s="25" t="s">
         <v>292</v>
@@ -9738,7 +9728,7 @@
         <v>115</v>
       </c>
       <c r="I151" s="2" t="s">
-        <v>1061</v>
+        <v>1059</v>
       </c>
       <c r="J151" s="6" t="s">
         <v>631</v>
@@ -9762,7 +9752,7 @@
         <v>232</v>
       </c>
       <c r="E152" s="9" t="s">
-        <v>910</v>
+        <v>908</v>
       </c>
       <c r="F152" s="25" t="s">
         <v>247</v>
@@ -9777,7 +9767,7 @@
         <v>590</v>
       </c>
       <c r="J152" s="6" t="s">
-        <v>1100</v>
+        <v>1098</v>
       </c>
       <c r="K152" s="5" t="s">
         <v>454</v>
@@ -9799,13 +9789,13 @@
         <v>109</v>
       </c>
       <c r="E153" s="9" t="s">
-        <v>911</v>
+        <v>909</v>
       </c>
       <c r="F153" s="25" t="s">
         <v>676</v>
       </c>
       <c r="G153" s="2" t="s">
-        <v>985</v>
+        <v>983</v>
       </c>
       <c r="H153" s="2" t="s">
         <v>108</v>
@@ -9836,13 +9826,13 @@
         <v>154</v>
       </c>
       <c r="E154" s="9" t="s">
-        <v>912</v>
+        <v>910</v>
       </c>
       <c r="F154" s="25" t="s">
         <v>278</v>
       </c>
       <c r="G154" s="2" t="s">
-        <v>986</v>
+        <v>984</v>
       </c>
       <c r="H154" s="2" t="s">
         <v>153</v>
@@ -9873,7 +9863,7 @@
         <v>57</v>
       </c>
       <c r="E155" s="9" t="s">
-        <v>913</v>
+        <v>911</v>
       </c>
       <c r="F155" s="26" t="s">
         <v>687</v>
@@ -9885,7 +9875,7 @@
         <v>56</v>
       </c>
       <c r="I155" s="12" t="s">
-        <v>1062</v>
+        <v>1060</v>
       </c>
       <c r="J155" s="1" t="s">
         <v>178</v>
@@ -9910,7 +9900,7 @@
         <v>8</v>
       </c>
       <c r="E156" s="37" t="s">
-        <v>914</v>
+        <v>912</v>
       </c>
       <c r="F156" s="26" t="s">
         <v>314</v>
@@ -9919,10 +9909,10 @@
         <v>7</v>
       </c>
       <c r="H156" s="38" t="s">
-        <v>1155</v>
+        <v>1153</v>
       </c>
       <c r="I156" s="33" t="s">
-        <v>1101</v>
+        <v>1099</v>
       </c>
       <c r="J156" s="36" t="s">
         <v>2</v>
@@ -9947,7 +9937,7 @@
         <v>11</v>
       </c>
       <c r="E157" s="9" t="s">
-        <v>915</v>
+        <v>913</v>
       </c>
       <c r="F157" s="26" t="s">
         <v>663</v>
@@ -9956,7 +9946,7 @@
         <v>16</v>
       </c>
       <c r="H157" s="12" t="s">
-        <v>969</v>
+        <v>967</v>
       </c>
       <c r="I157" s="12" t="s">
         <v>15</v>
@@ -9984,7 +9974,7 @@
         <v>11</v>
       </c>
       <c r="E158" s="9" t="s">
-        <v>916</v>
+        <v>914</v>
       </c>
       <c r="F158" s="26" t="s">
         <v>312</v>
@@ -9999,7 +9989,7 @@
         <v>664</v>
       </c>
       <c r="J158" s="1" t="s">
-        <v>971</v>
+        <v>969</v>
       </c>
       <c r="K158" s="5" t="s">
         <v>454</v>
@@ -10021,13 +10011,13 @@
         <v>11</v>
       </c>
       <c r="E159" s="9" t="s">
-        <v>917</v>
+        <v>915</v>
       </c>
       <c r="F159" s="26" t="s">
         <v>313</v>
       </c>
       <c r="G159" s="12" t="s">
-        <v>987</v>
+        <v>985</v>
       </c>
       <c r="H159" s="12" t="s">
         <v>13</v>
@@ -10058,7 +10048,7 @@
         <v>106</v>
       </c>
       <c r="E160" s="9" t="s">
-        <v>918</v>
+        <v>916</v>
       </c>
       <c r="F160" s="26" t="s">
         <v>572</v>
@@ -10070,7 +10060,7 @@
         <v>487</v>
       </c>
       <c r="I160" s="12" t="s">
-        <v>1063</v>
+        <v>1061</v>
       </c>
       <c r="J160" s="1" t="s">
         <v>489</v>
@@ -10095,7 +10085,7 @@
         <v>42</v>
       </c>
       <c r="E161" s="9" t="s">
-        <v>919</v>
+        <v>917</v>
       </c>
       <c r="F161" s="26" t="s">
         <v>308</v>
@@ -10110,7 +10100,7 @@
         <v>653</v>
       </c>
       <c r="J161" s="1" t="s">
-        <v>1102</v>
+        <v>1100</v>
       </c>
       <c r="K161" s="5" t="s">
         <v>454</v>
@@ -10132,7 +10122,7 @@
         <v>37</v>
       </c>
       <c r="E162" s="9" t="s">
-        <v>920</v>
+        <v>918</v>
       </c>
       <c r="F162" s="26" t="s">
         <v>309</v>
@@ -10144,7 +10134,7 @@
         <v>39</v>
       </c>
       <c r="I162" s="12" t="s">
-        <v>1064</v>
+        <v>1062</v>
       </c>
       <c r="J162" s="1" t="s">
         <v>659</v>
@@ -10166,13 +10156,13 @@
         <v>14</v>
       </c>
       <c r="D163" s="11" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="E163" s="9" t="s">
-        <v>921</v>
+        <v>919</v>
       </c>
       <c r="F163" s="26" t="s">
-        <v>1122</v>
+        <v>1120</v>
       </c>
       <c r="G163" s="12" t="s">
         <v>358</v>
@@ -10184,7 +10174,7 @@
         <v>360</v>
       </c>
       <c r="J163" s="1" t="s">
-        <v>1103</v>
+        <v>1101</v>
       </c>
       <c r="K163" s="5" t="s">
         <v>454</v>
@@ -10206,7 +10196,7 @@
         <v>36</v>
       </c>
       <c r="E164" s="9" t="s">
-        <v>922</v>
+        <v>920</v>
       </c>
       <c r="F164" s="26" t="s">
         <v>310</v>
@@ -10218,7 +10208,7 @@
         <v>35</v>
       </c>
       <c r="I164" s="12" t="s">
-        <v>1065</v>
+        <v>1063</v>
       </c>
       <c r="J164" s="1" t="s">
         <v>613</v>
@@ -10242,7 +10232,7 @@
         <v>60</v>
       </c>
       <c r="E165" s="9" t="s">
-        <v>923</v>
+        <v>921</v>
       </c>
       <c r="F165" s="25" t="s">
         <v>256</v>
@@ -10251,7 +10241,7 @@
         <v>217</v>
       </c>
       <c r="H165" s="2" t="s">
-        <v>1025</v>
+        <v>1023</v>
       </c>
       <c r="I165" s="2" t="s">
         <v>673</v>
@@ -10279,7 +10269,7 @@
         <v>60</v>
       </c>
       <c r="E166" s="9" t="s">
-        <v>924</v>
+        <v>922</v>
       </c>
       <c r="F166" s="25" t="s">
         <v>267</v>
@@ -10288,7 +10278,7 @@
         <v>185</v>
       </c>
       <c r="H166" s="2" t="s">
-        <v>1026</v>
+        <v>1024</v>
       </c>
       <c r="I166" s="2" t="s">
         <v>184</v>
@@ -10316,7 +10306,7 @@
         <v>60</v>
       </c>
       <c r="E167" s="9" t="s">
-        <v>925</v>
+        <v>923</v>
       </c>
       <c r="F167" s="25" t="s">
         <v>272</v>
@@ -10328,7 +10318,7 @@
         <v>612</v>
       </c>
       <c r="I167" s="6" t="s">
-        <v>1104</v>
+        <v>1102</v>
       </c>
       <c r="J167" s="2" t="s">
         <v>2</v>
@@ -10352,7 +10342,7 @@
         <v>60</v>
       </c>
       <c r="E168" s="9" t="s">
-        <v>926</v>
+        <v>924</v>
       </c>
       <c r="F168" s="25" t="s">
         <v>304</v>
@@ -10364,7 +10354,7 @@
         <v>63</v>
       </c>
       <c r="I168" s="2" t="s">
-        <v>1066</v>
+        <v>1064</v>
       </c>
       <c r="J168" s="6" t="s">
         <v>653</v>
@@ -10385,16 +10375,16 @@
         <v>14</v>
       </c>
       <c r="D169" s="11" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="E169" s="9" t="s">
-        <v>927</v>
+        <v>925</v>
       </c>
       <c r="F169" s="26" t="s">
-        <v>1124</v>
+        <v>1122</v>
       </c>
       <c r="G169" s="12" t="s">
-        <v>988</v>
+        <v>986</v>
       </c>
       <c r="H169" s="12" t="s">
         <v>490</v>
@@ -10425,7 +10415,7 @@
         <v>58</v>
       </c>
       <c r="E170" s="9" t="s">
-        <v>928</v>
+        <v>926</v>
       </c>
       <c r="F170" s="26" t="s">
         <v>697</v>
@@ -10459,10 +10449,10 @@
         <v>14</v>
       </c>
       <c r="D171" s="11" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="E171" s="9" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
       <c r="F171" s="26" t="s">
         <v>556</v>
@@ -10477,7 +10467,7 @@
         <v>381</v>
       </c>
       <c r="J171" s="1" t="s">
-        <v>1105</v>
+        <v>1103</v>
       </c>
       <c r="K171" s="5" t="s">
         <v>454</v>
@@ -10499,13 +10489,13 @@
         <v>106</v>
       </c>
       <c r="E172" s="16" t="s">
-        <v>930</v>
+        <v>928</v>
       </c>
       <c r="F172" s="27" t="s">
         <v>543</v>
       </c>
       <c r="G172" s="17" t="s">
-        <v>989</v>
+        <v>987</v>
       </c>
       <c r="H172" s="17" t="s">
         <v>347</v>
@@ -10536,13 +10526,13 @@
         <v>154</v>
       </c>
       <c r="E173" s="15" t="s">
-        <v>931</v>
+        <v>929</v>
       </c>
       <c r="F173" s="28" t="s">
         <v>539</v>
       </c>
       <c r="G173" s="14" t="s">
-        <v>990</v>
+        <v>988</v>
       </c>
       <c r="H173" s="14" t="s">
         <v>329</v>
@@ -10570,10 +10560,10 @@
         <v>14</v>
       </c>
       <c r="D174" s="11" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="E174" s="9" t="s">
-        <v>932</v>
+        <v>930</v>
       </c>
       <c r="F174" s="26" t="s">
         <v>542</v>
@@ -10582,7 +10572,7 @@
         <v>341</v>
       </c>
       <c r="H174" s="12" t="s">
-        <v>1027</v>
+        <v>1025</v>
       </c>
       <c r="I174" s="12" t="s">
         <v>342</v>
@@ -10607,13 +10597,13 @@
         <v>14</v>
       </c>
       <c r="D175" s="11" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="E175" s="37" t="s">
-        <v>933</v>
+        <v>931</v>
       </c>
       <c r="F175" s="32" t="s">
-        <v>1157</v>
+        <v>1155</v>
       </c>
       <c r="G175" s="12" t="s">
         <v>344</v>
@@ -10644,10 +10634,10 @@
         <v>14</v>
       </c>
       <c r="D176" s="11" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E176" s="9" t="s">
-        <v>934</v>
+        <v>932</v>
       </c>
       <c r="F176" s="26" t="s">
         <v>569</v>
@@ -10656,7 +10646,7 @@
         <v>455</v>
       </c>
       <c r="H176" s="1" t="s">
-        <v>1028</v>
+        <v>1026</v>
       </c>
       <c r="I176" s="12" t="s">
         <v>456</v>
@@ -10684,7 +10674,7 @@
         <v>103</v>
       </c>
       <c r="E177" s="9" t="s">
-        <v>935</v>
+        <v>933</v>
       </c>
       <c r="F177" s="25" t="s">
         <v>262</v>
@@ -10693,7 +10683,7 @@
         <v>198</v>
       </c>
       <c r="H177" s="2" t="s">
-        <v>1029</v>
+        <v>1027</v>
       </c>
       <c r="I177" s="2" t="s">
         <v>197</v>
@@ -10721,7 +10711,7 @@
         <v>50</v>
       </c>
       <c r="E178" s="9" t="s">
-        <v>936</v>
+        <v>934</v>
       </c>
       <c r="F178" s="26" t="s">
         <v>306</v>
@@ -10736,7 +10726,7 @@
         <v>656</v>
       </c>
       <c r="J178" s="1" t="s">
-        <v>1094</v>
+        <v>1092</v>
       </c>
       <c r="K178" s="5" t="s">
         <v>454</v>
@@ -10755,13 +10745,13 @@
         <v>14</v>
       </c>
       <c r="D179" s="11" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="E179" s="9" t="s">
-        <v>937</v>
+        <v>935</v>
       </c>
       <c r="F179" s="26" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="G179" s="12" t="s">
         <v>368</v>
@@ -10773,7 +10763,7 @@
         <v>370</v>
       </c>
       <c r="J179" s="1" t="s">
-        <v>1106</v>
+        <v>1104</v>
       </c>
       <c r="K179" s="5" t="s">
         <v>454</v>
@@ -10792,10 +10782,10 @@
         <v>14</v>
       </c>
       <c r="D180" s="11" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="E180" s="9" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="F180" s="26" t="s">
         <v>696</v>
@@ -10807,7 +10797,7 @@
         <v>371</v>
       </c>
       <c r="I180" s="12" t="s">
-        <v>1067</v>
+        <v>1065</v>
       </c>
       <c r="J180" s="1" t="s">
         <v>373</v>
@@ -10832,13 +10822,13 @@
         <v>73</v>
       </c>
       <c r="E181" s="9" t="s">
-        <v>939</v>
+        <v>937</v>
       </c>
       <c r="F181" s="26" t="s">
-        <v>1125</v>
+        <v>1123</v>
       </c>
       <c r="G181" s="12" t="s">
-        <v>991</v>
+        <v>989</v>
       </c>
       <c r="H181" s="12" t="s">
         <v>374</v>
@@ -10869,7 +10859,7 @@
         <v>25</v>
       </c>
       <c r="E182" s="9" t="s">
-        <v>940</v>
+        <v>938</v>
       </c>
       <c r="F182" s="26" t="s">
         <v>689</v>
@@ -10903,10 +10893,10 @@
         <v>14</v>
       </c>
       <c r="D183" s="11" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="E183" s="9" t="s">
-        <v>941</v>
+        <v>939</v>
       </c>
       <c r="F183" s="26" t="s">
         <v>698</v>
@@ -10918,7 +10908,7 @@
         <v>392</v>
       </c>
       <c r="I183" s="12" t="s">
-        <v>1068</v>
+        <v>1066</v>
       </c>
       <c r="J183" s="1" t="s">
         <v>394</v>
@@ -10943,7 +10933,7 @@
         <v>148</v>
       </c>
       <c r="E184" s="9" t="s">
-        <v>942</v>
+        <v>940</v>
       </c>
       <c r="F184" s="26" t="s">
         <v>559</v>
@@ -10952,7 +10942,7 @@
         <v>403</v>
       </c>
       <c r="H184" s="12" t="s">
-        <v>1030</v>
+        <v>1028</v>
       </c>
       <c r="I184" s="12" t="s">
         <v>404</v>
@@ -10980,10 +10970,10 @@
         <v>73</v>
       </c>
       <c r="E185" s="9" t="s">
-        <v>943</v>
+        <v>941</v>
       </c>
       <c r="F185" s="26" t="s">
-        <v>1126</v>
+        <v>1124</v>
       </c>
       <c r="G185" s="12" t="s">
         <v>412</v>
@@ -10995,7 +10985,7 @@
         <v>414</v>
       </c>
       <c r="J185" s="1" t="s">
-        <v>1107</v>
+        <v>1105</v>
       </c>
       <c r="K185" s="5" t="s">
         <v>454</v>
@@ -11017,7 +11007,7 @@
         <v>58</v>
       </c>
       <c r="E186" s="9" t="s">
-        <v>944</v>
+        <v>942</v>
       </c>
       <c r="F186" s="26" t="s">
         <v>700</v>
@@ -11026,7 +11016,7 @@
         <v>416</v>
       </c>
       <c r="H186" s="12" t="s">
-        <v>1031</v>
+        <v>1029</v>
       </c>
       <c r="I186" s="12" t="s">
         <v>417</v>
@@ -11054,10 +11044,10 @@
         <v>19</v>
       </c>
       <c r="E187" s="9" t="s">
-        <v>945</v>
+        <v>943</v>
       </c>
       <c r="F187" s="29" t="s">
-        <v>1127</v>
+        <v>1125</v>
       </c>
       <c r="G187" s="1" t="s">
         <v>24</v>
@@ -11066,7 +11056,7 @@
         <v>83</v>
       </c>
       <c r="I187" s="1" t="s">
-        <v>1069</v>
+        <v>1067</v>
       </c>
       <c r="J187" s="1" t="s">
         <v>2</v>
@@ -11091,22 +11081,22 @@
         <v>19</v>
       </c>
       <c r="E188" s="9" t="s">
-        <v>946</v>
+        <v>944</v>
       </c>
       <c r="F188" s="29" t="s">
-        <v>1128</v>
+        <v>1126</v>
       </c>
       <c r="G188" s="1" t="s">
+        <v>737</v>
+      </c>
+      <c r="H188" s="1" t="s">
+        <v>1030</v>
+      </c>
+      <c r="I188" s="1" t="s">
+        <v>738</v>
+      </c>
+      <c r="J188" s="1" t="s">
         <v>739</v>
-      </c>
-      <c r="H188" s="1" t="s">
-        <v>1032</v>
-      </c>
-      <c r="I188" s="1" t="s">
-        <v>740</v>
-      </c>
-      <c r="J188" s="1" t="s">
-        <v>741</v>
       </c>
       <c r="K188" s="5" t="s">
         <v>452</v>
@@ -11125,25 +11115,25 @@
         <v>14</v>
       </c>
       <c r="D189" s="4" t="s">
-        <v>756</v>
+        <v>754</v>
       </c>
       <c r="E189" s="9" t="s">
-        <v>947</v>
+        <v>945</v>
       </c>
       <c r="F189" s="29" t="s">
-        <v>1129</v>
+        <v>1127</v>
       </c>
       <c r="G189" s="1" t="s">
+        <v>740</v>
+      </c>
+      <c r="H189" s="1" t="s">
+        <v>1031</v>
+      </c>
+      <c r="I189" s="1" t="s">
+        <v>741</v>
+      </c>
+      <c r="J189" s="1" t="s">
         <v>742</v>
-      </c>
-      <c r="H189" s="1" t="s">
-        <v>1033</v>
-      </c>
-      <c r="I189" s="1" t="s">
-        <v>743</v>
-      </c>
-      <c r="J189" s="1" t="s">
-        <v>744</v>
       </c>
       <c r="K189" s="5" t="s">
         <v>452</v>
@@ -11162,25 +11152,25 @@
         <v>14</v>
       </c>
       <c r="D190" s="4" t="s">
-        <v>756</v>
+        <v>754</v>
       </c>
       <c r="E190" s="9" t="s">
-        <v>948</v>
+        <v>946</v>
       </c>
       <c r="F190" s="29" t="s">
+        <v>743</v>
+      </c>
+      <c r="G190" s="1" t="s">
+        <v>744</v>
+      </c>
+      <c r="H190" s="1" t="s">
         <v>745</v>
       </c>
-      <c r="G190" s="1" t="s">
+      <c r="I190" s="1" t="s">
+        <v>1068</v>
+      </c>
+      <c r="J190" s="1" t="s">
         <v>746</v>
-      </c>
-      <c r="H190" s="1" t="s">
-        <v>747</v>
-      </c>
-      <c r="I190" s="1" t="s">
-        <v>1070</v>
-      </c>
-      <c r="J190" s="1" t="s">
-        <v>748</v>
       </c>
       <c r="K190" s="5" t="s">
         <v>451</v>
@@ -11199,25 +11189,25 @@
         <v>14</v>
       </c>
       <c r="D191" s="4" t="s">
-        <v>757</v>
+        <v>755</v>
       </c>
       <c r="E191" s="9" t="s">
-        <v>949</v>
+        <v>947</v>
       </c>
       <c r="F191" s="29" t="s">
+        <v>747</v>
+      </c>
+      <c r="G191" s="1" t="s">
+        <v>990</v>
+      </c>
+      <c r="H191" s="1" t="s">
+        <v>748</v>
+      </c>
+      <c r="I191" s="1" t="s">
         <v>749</v>
       </c>
-      <c r="G191" s="1" t="s">
-        <v>992</v>
-      </c>
-      <c r="H191" s="1" t="s">
+      <c r="J191" s="1" t="s">
         <v>750</v>
-      </c>
-      <c r="I191" s="1" t="s">
-        <v>751</v>
-      </c>
-      <c r="J191" s="1" t="s">
-        <v>752</v>
       </c>
       <c r="K191" s="5" t="s">
         <v>453</v>
@@ -11239,19 +11229,19 @@
         <v>78</v>
       </c>
       <c r="E192" s="9" t="s">
-        <v>950</v>
+        <v>948</v>
       </c>
       <c r="F192" s="30" t="s">
-        <v>755</v>
+        <v>753</v>
       </c>
       <c r="G192" s="6" t="s">
-        <v>993</v>
+        <v>991</v>
       </c>
       <c r="H192" s="6" t="s">
-        <v>754</v>
+        <v>752</v>
       </c>
       <c r="I192" s="6" t="s">
-        <v>753</v>
+        <v>751</v>
       </c>
       <c r="J192" s="6" t="s">
         <v>2</v>
@@ -11274,119 +11264,156 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D85EA40A-B229-42D6-900A-3C11C6DED23E}">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:13" s="3" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A1" s="4">
+    <row r="1" spans="1:13" s="3" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
+        <v>244</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>465</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>757</v>
+      </c>
+      <c r="F1" s="24" t="s">
+        <v>756</v>
+      </c>
+      <c r="G1" s="13" t="s">
+        <v>471</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>472</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>474</v>
+      </c>
+      <c r="J1" s="10" t="s">
+        <v>473</v>
+      </c>
+      <c r="K1" s="13" t="s">
+        <v>705</v>
+      </c>
+      <c r="L1" s="13"/>
+      <c r="M1" s="13"/>
+    </row>
+    <row r="2" spans="1:13" s="3" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A2" s="4">
         <v>96</v>
       </c>
-      <c r="B1" s="9">
-        <v>1</v>
-      </c>
-      <c r="C1" s="11" t="s">
+      <c r="B2" s="9">
+        <v>1</v>
+      </c>
+      <c r="C2" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="11" t="s">
-        <v>716</v>
-      </c>
-      <c r="E1" s="9" t="s">
-        <v>855</v>
-      </c>
-      <c r="F1" s="26" t="s">
-        <v>1111</v>
-      </c>
-      <c r="G1" s="12" t="s">
-        <v>973</v>
-      </c>
-      <c r="H1" s="12" t="s">
+      <c r="D2" s="11" t="s">
+        <v>715</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>853</v>
+      </c>
+      <c r="F2" s="26" t="s">
+        <v>1109</v>
+      </c>
+      <c r="G2" s="12" t="s">
+        <v>971</v>
+      </c>
+      <c r="H2" s="12" t="s">
         <v>553</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>554</v>
       </c>
-      <c r="J1" s="12" t="s">
+      <c r="J2" s="12" t="s">
         <v>555</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="K2" s="5" t="s">
         <v>453</v>
-      </c>
-      <c r="L1"/>
-      <c r="M1"/>
-    </row>
-    <row r="2" spans="1:13" s="3" customFormat="1" ht="72" x14ac:dyDescent="0.3">
-      <c r="A2" s="4">
-        <v>95</v>
-      </c>
-      <c r="B2" s="9">
-        <v>1</v>
-      </c>
-      <c r="C2" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" s="11" t="s">
-        <v>713</v>
-      </c>
-      <c r="E2" s="9" t="s">
-        <v>854</v>
-      </c>
-      <c r="F2" s="26" t="s">
-        <v>1112</v>
-      </c>
-      <c r="G2" s="12" t="s">
-        <v>546</v>
-      </c>
-      <c r="H2" s="12" t="s">
-        <v>547</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="J2" s="12" t="s">
-        <v>1086</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>454</v>
       </c>
       <c r="L2"/>
       <c r="M2"/>
     </row>
-    <row r="3" spans="1:13" s="3" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" s="3" customFormat="1" ht="72" x14ac:dyDescent="0.3">
       <c r="A3" s="4">
-        <v>163</v>
+        <v>95</v>
       </c>
       <c r="B3" s="9">
         <v>1</v>
       </c>
-      <c r="C3" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>10</v>
+      <c r="C3" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>712</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>922</v>
+        <v>852</v>
       </c>
       <c r="F3" s="26" t="s">
-        <v>1123</v>
+        <v>1110</v>
       </c>
       <c r="G3" s="12" t="s">
-        <v>218</v>
+        <v>546</v>
       </c>
       <c r="H3" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="I3" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="J3" s="1" t="s">
+        <v>547</v>
+      </c>
+      <c r="I3" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="J3" s="12" t="s">
+        <v>1084</v>
+      </c>
       <c r="K3" s="5" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="L3"/>
       <c r="M3"/>
+    </row>
+    <row r="4" spans="1:13" s="3" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A4" s="4">
+        <v>163</v>
+      </c>
+      <c r="B4" s="9">
+        <v>1</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>920</v>
+      </c>
+      <c r="F4" s="26" t="s">
+        <v>1121</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>218</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="I4" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>451</v>
+      </c>
+      <c r="L4"/>
+      <c r="M4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>